<commit_message>
docs(repo): ceremonias, métricas y retrospectiva del Sprint 1 (#35)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -1147,7 +1147,7 @@
         <v>46301</v>
       </c>
       <c r="D3" s="13">
-        <v>46302</v>
+        <v>46305</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>42</v>
@@ -1206,11 +1206,9 @@
         <v>43</v>
       </c>
       <c r="C4" s="13">
-        <v>46303</v>
-      </c>
-      <c r="D4" s="13">
-        <v>46305</v>
-      </c>
+        <v>46306</v>
+      </c>
+      <c r="D4" s="13"/>
       <c r="E4" s="14" t="s">
         <v>44</v>
       </c>
@@ -1454,10 +1452,14 @@
         <v>1</v>
       </c>
       <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="G2" s="27">
+        <v>46302.973519</v>
+      </c>
       <c r="H2" s="27"/>
       <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
+      <c r="J2" s="27">
+        <v>46304.618704</v>
+      </c>
       <c r="K2" s="26">
         <v>0</v>
       </c>
@@ -1470,7 +1472,11 @@
       <c r="N2" s="17">
         <f>IF(AND(ISNUMBER(J2),ISNUMBER(G2)),J2-G2,"")</f>
       </c>
-      <c r="O2" s="14"/>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>Registrado el 2026-10-10 en la #35: durante el sprint no se anotaron las fechas. En análisis = primer commit de #23 (PR #54), la fecha más probable. Done = cierre real de #11. Ready, En atención y En validación no se registraron.</t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1489,10 +1495,14 @@
         <v>1</v>
       </c>
       <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
+      <c r="G3" s="27">
+        <v>46303.871377</v>
+      </c>
       <c r="H3" s="27"/>
       <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
+      <c r="J3" s="27">
+        <v>46305.83897</v>
+      </c>
       <c r="K3" s="26">
         <v>0</v>
       </c>
@@ -1505,7 +1515,11 @@
       <c r="N3" s="17">
         <f>IF(AND(ISNUMBER(J3),ISNUMBER(G3)),J3-G3,"")</f>
       </c>
-      <c r="O3" s="14"/>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Registrado el 2026-10-10 en la #35: durante el sprint no se anotaron las fechas. En análisis = primer commit de #26 (PR #55), la fecha más probable. Done = cierre real de #12. Ready, En atención y En validación no se registraron.</t>
+        </is>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -1524,10 +1538,14 @@
         <v>1</v>
       </c>
       <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="G4" s="27">
+        <v>46303.879896</v>
+      </c>
       <c r="H4" s="27"/>
       <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="J4" s="27">
+        <v>46305.839016</v>
+      </c>
       <c r="K4" s="26">
         <v>0</v>
       </c>
@@ -1540,7 +1558,11 @@
       <c r="N4" s="17">
         <f>IF(AND(ISNUMBER(J4),ISNUMBER(G4)),J4-G4,"")</f>
       </c>
-      <c r="O4" s="14"/>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>Registrado el 2026-10-10 en la #35: durante el sprint no se anotaron las fechas. En análisis = primer commit de #29 (PR #58), la fecha más probable. Done = cierre real de #13. Ready, En atención y En validación no se registraron.</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1594,10 +1616,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
+      <c r="G6" s="27">
+        <v>46304.487975</v>
+      </c>
       <c r="H6" s="27"/>
       <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="J6" s="27">
+        <v>46305.874826</v>
+      </c>
       <c r="K6" s="26">
         <v>0</v>
       </c>
@@ -1610,7 +1636,11 @@
       <c r="N6" s="17">
         <f>IF(AND(ISNUMBER(J6),ISNUMBER(G6)),J6-G6,"")</f>
       </c>
-      <c r="O6" s="14"/>
+      <c r="O6" s="14" t="inlineStr">
+        <is>
+          <t>Registrado el 2026-10-10 en la #35: durante el sprint no se anotaron las fechas. En análisis = primer commit de #32 (PR #61), la fecha más probable. Done = cierre real de #15. Ready, En atención y En validación no se registraron.</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -4091,19 +4121,65 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="26"/>
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>DEF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="26">
+        <v>1</v>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>HU-02, HU-03, HU-05</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Tildes corruptas al cargar schema.sql y seeds.sql en Windows: falta SET NAMES utf8mb4 y el ENUM caso.estado queda mal guardado.</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>1. Cargar db/schema.sql y db/seeds.sql con el cliente mysql de Windows, sin --default-character-set. 2. SELECT @@character_set_client (cp850). 3. Consultar usuario 1 y SHOW COLUMNS de caso.estado.</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Laura Gómez y los valores del ENUM estado con tildes correctas.</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Nombres corruptos (Laura G├│mez) y ENUM estado corrupto: el cambio a En análisis fallaría (rompe CP-04).</t>
+        </is>
+      </c>
+      <c r="I2" s="26" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J2" s="26" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K2" s="27">
+        <v>46303.941852</v>
+      </c>
+      <c r="L2" s="27">
+        <v>46304.520359</v>
+      </c>
+      <c r="M2" s="26" t="inlineStr">
+        <is>
+          <t>CP-04</t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="26"/>

</xml_diff>

<commit_message>
docs(repo): Sprint 2 Planning, fechas replanificadas y decisión de HU-04 (#36)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -1208,7 +1208,9 @@
       <c r="C4" s="13">
         <v>46306</v>
       </c>
-      <c r="D4" s="13"/>
+      <c r="D4" s="13">
+        <v>46306</v>
+      </c>
       <c r="E4" s="14" t="s">
         <v>44</v>
       </c>
@@ -1266,7 +1268,7 @@
         <v>45</v>
       </c>
       <c r="C5" s="13">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="D5" s="13">
         <v>46307</v>

</xml_diff>

<commit_message>
docs(repo): Sprint 3 Planning y refinamiento de HU-09, 10, 11 y 12 (#37)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -20,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy hh:mm"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd hh:mm"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -86,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -139,6 +140,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -236,7 +238,12 @@
     </comment>
     <comment ref="C5" authorId="0" shapeId="0">
       <text>
-        <t>Plan: 12 oct. Se corre al 13 porque el Sprint 2 terminó el 12; confirmar en la #37.</t>
+        <t>Plan original: 11–12 oct. Empieza en el Sprint 3 Planning (2026-10-12 22:24, creación de #97). Lleva la hora para no contar en el Sprint 3 las HU del Sprint 2, que llegaron a Done el 12 oct antes de las 21:33. Registrado en la #37.</t>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0">
+      <text>
+        <t>Fin: 13 oct, día de la entrega. Registrado en la #37.</t>
       </text>
     </comment>
   </commentList>
@@ -1140,8 +1147,8 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>46308</v>
+      <c r="C5" s="27" t="n">
+        <v>46307.93368055556</v>
       </c>
       <c r="D5" s="13" t="n">
         <v>46308</v>
@@ -1822,7 +1829,9 @@
       <c r="E10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="27" t="n"/>
+      <c r="F10" s="27" t="n">
+        <v>46307.93368055556</v>
+      </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" s="27" t="n"/>
       <c r="I10" s="27" t="n"/>
@@ -1842,7 +1851,11 @@
         <f>IF(AND(ISNUMBER(J10),ISNUMBER(G10)),J10-G10,"")</f>
         <v/>
       </c>
-      <c r="O10" s="14" t="n"/>
+      <c r="O10" s="14" t="inlineStr">
+        <is>
+          <t>Ready = creación de las sub-issues (#97, #98 y #99) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1866,7 +1879,9 @@
       <c r="E11" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="27" t="n"/>
+      <c r="F11" s="27" t="n">
+        <v>46307.93414351852</v>
+      </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" s="27" t="n"/>
       <c r="I11" s="27" t="n"/>
@@ -1886,7 +1901,11 @@
         <f>IF(AND(ISNUMBER(J11),ISNUMBER(G11)),J11-G11,"")</f>
         <v/>
       </c>
-      <c r="O11" s="14" t="n"/>
+      <c r="O11" s="14" t="inlineStr">
+        <is>
+          <t>Ready = creación de las sub-issues (#100, #101 y #102) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1910,7 +1929,9 @@
       <c r="E12" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="27" t="n"/>
+      <c r="F12" s="27" t="n">
+        <v>46307.93440972222</v>
+      </c>
       <c r="G12" s="27" t="n"/>
       <c r="H12" s="27" t="n"/>
       <c r="I12" s="27" t="n"/>
@@ -1930,7 +1951,11 @@
         <f>IF(AND(ISNUMBER(J12),ISNUMBER(G12)),J12-G12,"")</f>
         <v/>
       </c>
-      <c r="O12" s="14" t="n"/>
+      <c r="O12" s="14" t="inlineStr">
+        <is>
+          <t>Ready = creación de las sub-issues (#103, #104 y #105) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1954,7 +1979,9 @@
       <c r="E13" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="27" t="n"/>
+      <c r="F13" s="27" t="n">
+        <v>46307.93466435185</v>
+      </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" s="27" t="n"/>
       <c r="I13" s="27" t="n"/>
@@ -1974,7 +2001,11 @@
         <f>IF(AND(ISNUMBER(J13),ISNUMBER(G13)),J13-G13,"")</f>
         <v/>
       </c>
-      <c r="O13" s="14" t="n"/>
+      <c r="O13" s="14" t="inlineStr">
+        <is>
+          <t>Ready = creación de las sub-issues (#106, #107 y #108) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
docs(repo): ceremonias, métricas y retrospectiva del Sprint 3 (#37)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="12000" windowHeight="24000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen por sprint" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WIP diario" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloqueos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen por sprint" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Historias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="WIP diario" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bloqueos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Defectos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -1832,10 +1832,14 @@
       <c r="F10" s="27" t="n">
         <v>46307.93368055556</v>
       </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="27" t="n">
+        <v>46308.13244212963</v>
+      </c>
       <c r="H10" s="27" t="n"/>
       <c r="I10" s="27" t="n"/>
-      <c r="J10" s="27" t="n"/>
+      <c r="J10" s="27" t="n">
+        <v>46308.36922453704</v>
+      </c>
       <c r="K10" s="26" t="n">
         <v>0</v>
       </c>
@@ -1853,7 +1857,7 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Ready = creación de las sub-issues (#97, #98 y #99) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+          <t>Ready = creación de las sub-issues (#97, #98 y #99) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37. Registrado el 2026-10-13 en la #37: durante el sprint no se anotaron las demás fechas. En análisis = primer commit de #97 (PR #111), la fecha más probable. Done = cierre real de #19. En atención y En validación no se registraron.</t>
         </is>
       </c>
     </row>
@@ -1882,10 +1886,14 @@
       <c r="F11" s="27" t="n">
         <v>46307.93414351852</v>
       </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="27" t="n">
+        <v>46308.13940972222</v>
+      </c>
       <c r="H11" s="27" t="n"/>
       <c r="I11" s="27" t="n"/>
-      <c r="J11" s="27" t="n"/>
+      <c r="J11" s="27" t="n">
+        <v>46308.37537037037</v>
+      </c>
       <c r="K11" s="26" t="n">
         <v>0</v>
       </c>
@@ -1903,7 +1911,7 @@
       </c>
       <c r="O11" s="14" t="inlineStr">
         <is>
-          <t>Ready = creación de las sub-issues (#100, #101 y #102) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+          <t>Ready = creación de las sub-issues (#100, #101 y #102) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37. Registrado el 2026-10-13 en la #37: durante el sprint no se anotaron las demás fechas. En análisis = primer commit de #100 (PR #112), la fecha más probable. Done = cierre real de #20. En atención y En validación no se registraron.</t>
         </is>
       </c>
     </row>
@@ -1932,10 +1940,14 @@
       <c r="F12" s="27" t="n">
         <v>46307.93440972222</v>
       </c>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="27" t="n">
+        <v>46308.1466087963</v>
+      </c>
       <c r="H12" s="27" t="n"/>
       <c r="I12" s="27" t="n"/>
-      <c r="J12" s="27" t="n"/>
+      <c r="J12" s="27" t="n">
+        <v>46308.44297453704</v>
+      </c>
       <c r="K12" s="26" t="n">
         <v>0</v>
       </c>
@@ -1953,7 +1965,7 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Ready = creación de las sub-issues (#103, #104 y #105) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+          <t>Ready = creación de las sub-issues (#103, #104 y #105) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37. Registrado el 2026-10-13 en la #37: durante el sprint no se anotaron las demás fechas. En análisis = primer commit de #103 (PR #113), la fecha más probable. Done = cierre real de #21. En atención y En validación no se registraron.</t>
         </is>
       </c>
     </row>
@@ -1982,10 +1994,14 @@
       <c r="F13" s="27" t="n">
         <v>46307.93466435185</v>
       </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="27" t="n">
+        <v>46308.15221064815</v>
+      </c>
       <c r="H13" s="27" t="n"/>
       <c r="I13" s="27" t="n"/>
-      <c r="J13" s="27" t="n"/>
+      <c r="J13" s="27" t="n">
+        <v>46308.44291666667</v>
+      </c>
       <c r="K13" s="26" t="n">
         <v>0</v>
       </c>
@@ -2003,7 +2019,7 @@
       </c>
       <c r="O13" s="14" t="inlineStr">
         <is>
-          <t>Ready = creación de las sub-issues (#106, #107 y #108) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37.</t>
+          <t>Ready = creación de las sub-issues (#106, #107 y #108) en el Sprint 3 Planning, 2026-10-12, con la ficha refinada en docs/historias/. Registrado en la #37. Registrado el 2026-10-13 en la #37: durante el sprint no se anotaron las demás fechas. En análisis = primer commit de #106 (PR #114), la fecha más probable. Done = cierre real de #22. En atención y En validación no se registraron.</t>
         </is>
       </c>
     </row>
@@ -4669,13 +4685,15 @@
       </c>
       <c r="J3" s="26" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K3" s="27" t="n">
         <v>46307.84027777778</v>
       </c>
-      <c r="L3" s="27" t="n"/>
+      <c r="L3" s="27" t="n">
+        <v>46308.30768518519</v>
+      </c>
       <c r="M3" s="26" t="inlineStr">
         <is>
           <t>HU-07 (QA de la #77)</t>

</xml_diff>

<commit_message>
docs(repo): registrar DEF-03 del detalle del caso (#37)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -4701,19 +4701,63 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="n"/>
-      <c r="B4" s="26" t="n"/>
-      <c r="C4" s="26" t="n"/>
-      <c r="D4" s="26" t="n"/>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="14" t="n"/>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
-      <c r="I4" s="26" t="n"/>
-      <c r="J4" s="26" t="n"/>
-      <c r="K4" s="27" t="n"/>
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>DEF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>HU-12</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>#123</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>La pantalla de detalle del caso muestra 'Caso no encontrado' ante cualquier error (500, fallo de red), no solo ante el 404.</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>1. Provocar un error del servidor: RENAME TABLE atencion TO atencion_x. 2. Con Laura Gómez abrir /mis-solicitudes/5. 3. Restaurar la tabla.</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>'Caso no encontrado' solo con el 404; en los demás casos, el mensaje de la API o 'No se pudo cargar el caso'.</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>La API responde 500 y la pantalla muestra 'Caso no encontrado', igual que con un caso inexistente o ajeno.</t>
+        </is>
+      </c>
+      <c r="I4" s="26" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J4" s="26" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="K4" s="27" t="n">
+        <v>46308.3612037037</v>
+      </c>
       <c r="L4" s="27" t="n"/>
-      <c r="M4" s="26" t="n"/>
+      <c r="M4" s="26" t="inlineStr">
+        <is>
+          <t>HU-12 (QA de la #108)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="26" t="n"/>

</xml_diff>

<commit_message>
docs(repo): cerrar DEF-03 en la hoja de defectos y las pruebas (#123)
</commit_message>
<xml_diff>
--- a/docs/metricas/seguimiento.xlsx
+++ b/docs/metricas/seguimiento.xlsx
@@ -4746,13 +4746,15 @@
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K4" s="27" t="n">
         <v>46308.3612037037</v>
       </c>
-      <c r="L4" s="27" t="n"/>
+      <c r="L4" s="27" t="n">
+        <v>46308.48283564814</v>
+      </c>
       <c r="M4" s="26" t="inlineStr">
         <is>
           <t>HU-12 (QA de la #108)</t>

</xml_diff>